<commit_message>
sudah templating strukturisasi file folder
</commit_message>
<xml_diff>
--- a/tools/Kendali Aplikasi Koperasi Ahmadi.xlsx
+++ b/tools/Kendali Aplikasi Koperasi Ahmadi.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\LARAGON\www\2026\5APKKOPERASIAHMADI\TOOLS\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\LARAGON\www\2026\5APKKOPERASIAHMADI\tools\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8984DEAB-49AD-4BB9-83AF-E8CFE60AC936}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B9AD044-C5F3-475A-883E-341DAE25D3E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PROTA REVISI" sheetId="5" r:id="rId1"/>
@@ -85,7 +85,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="602" uniqueCount="322">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="602" uniqueCount="323">
   <si>
     <t>BREAKDOWN FITUR PADA APLIKASI</t>
   </si>
@@ -1063,6 +1063,9 @@
   <si>
     <t>NIP. 19860505 201403 1 003</t>
   </si>
+  <si>
+    <t>: Ahmadi Muslim</t>
+  </si>
 </sst>
 </file>
 
@@ -1950,53 +1953,13 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="27" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="27" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="23" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="25" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="23" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="25" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="28" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="30" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="28" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="30" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="19" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="21" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="19" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="21" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="22" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="22" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="11" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -2034,13 +1997,53 @@
     <xf numFmtId="0" fontId="29" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="19" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="21" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="19" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="21" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="22" fillId="22" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="22" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="23" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="25" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="23" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="25" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="27" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="27" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="28" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="30" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="28" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="30" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2592,40 +2595,40 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:L134"/>
-  <sheetFormatPr defaultColWidth="12.5546875" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="11" style="38" customWidth="1"/>
-    <col min="2" max="2" width="17.109375" style="38" customWidth="1"/>
-    <col min="3" max="3" width="47.5546875" style="38" customWidth="1"/>
-    <col min="4" max="4" width="8.109375" style="38" customWidth="1"/>
-    <col min="5" max="5" width="9.33203125" style="38" customWidth="1"/>
+    <col min="2" max="2" width="17.140625" style="38" customWidth="1"/>
+    <col min="3" max="3" width="47.5703125" style="38" customWidth="1"/>
+    <col min="4" max="4" width="8.140625" style="38" customWidth="1"/>
+    <col min="5" max="5" width="9.28515625" style="38" customWidth="1"/>
     <col min="6" max="6" width="8" style="38" customWidth="1"/>
-    <col min="7" max="7" width="10.21875" style="38" customWidth="1"/>
+    <col min="7" max="7" width="10.28515625" style="38" customWidth="1"/>
     <col min="8" max="8" width="7" style="38" customWidth="1"/>
-    <col min="9" max="9" width="7.44140625" style="38" customWidth="1"/>
-    <col min="10" max="10" width="6.21875" style="38" customWidth="1"/>
-    <col min="11" max="11" width="7.44140625" style="38" customWidth="1"/>
-    <col min="12" max="12" width="6.44140625" style="110" customWidth="1"/>
-    <col min="13" max="16384" width="12.5546875" style="38"/>
+    <col min="9" max="9" width="7.42578125" style="38" customWidth="1"/>
+    <col min="10" max="10" width="6.28515625" style="38" customWidth="1"/>
+    <col min="11" max="11" width="7.42578125" style="38" customWidth="1"/>
+    <col min="12" max="12" width="6.42578125" style="110" customWidth="1"/>
+    <col min="13" max="16384" width="12.5703125" style="38"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="17.399999999999999">
-      <c r="A1" s="140" t="s">
+    <row r="1" spans="1:12" ht="18">
+      <c r="A1" s="114" t="s">
         <v>83</v>
       </c>
-      <c r="B1" s="140"/>
-      <c r="C1" s="140"/>
-      <c r="D1" s="140"/>
-      <c r="E1" s="140"/>
-      <c r="F1" s="140"/>
-      <c r="G1" s="140"/>
-      <c r="H1" s="140"/>
-      <c r="I1" s="140"/>
-      <c r="J1" s="140"/>
-      <c r="K1" s="140"/>
-      <c r="L1" s="140"/>
-    </row>
-    <row r="2" spans="1:12" ht="17.399999999999999">
+      <c r="B1" s="114"/>
+      <c r="C1" s="114"/>
+      <c r="D1" s="114"/>
+      <c r="E1" s="114"/>
+      <c r="F1" s="114"/>
+      <c r="G1" s="114"/>
+      <c r="H1" s="114"/>
+      <c r="I1" s="114"/>
+      <c r="J1" s="114"/>
+      <c r="K1" s="114"/>
+      <c r="L1" s="114"/>
+    </row>
+    <row r="2" spans="1:12" ht="18">
       <c r="A2" s="39"/>
       <c r="B2" s="39"/>
       <c r="C2" s="39"/>
@@ -2639,11 +2642,11 @@
       <c r="K2" s="40"/>
       <c r="L2" s="39"/>
     </row>
-    <row r="3" spans="1:12" ht="14.4">
-      <c r="A3" s="141" t="s">
+    <row r="3" spans="1:12" ht="15">
+      <c r="A3" s="112" t="s">
         <v>84</v>
       </c>
-      <c r="B3" s="142"/>
+      <c r="B3" s="113"/>
       <c r="C3" s="42" t="s">
         <v>85</v>
       </c>
@@ -2657,7 +2660,7 @@
       <c r="K3" s="40"/>
       <c r="L3" s="44"/>
     </row>
-    <row r="4" spans="1:12" ht="14.4">
+    <row r="4" spans="1:12" ht="15">
       <c r="A4" s="45" t="s">
         <v>86</v>
       </c>
@@ -2675,26 +2678,26 @@
       <c r="K4" s="40"/>
       <c r="L4" s="47"/>
     </row>
-    <row r="5" spans="1:12" ht="14.4">
+    <row r="5" spans="1:12" ht="15">
       <c r="A5" s="45" t="s">
         <v>88</v>
       </c>
       <c r="B5" s="45"/>
-      <c r="C5" s="143" t="s">
+      <c r="C5" s="115" t="s">
         <v>89</v>
       </c>
-      <c r="D5" s="142"/>
+      <c r="D5" s="113"/>
       <c r="H5" s="43"/>
       <c r="I5" s="40"/>
       <c r="J5" s="40"/>
       <c r="K5" s="40"/>
       <c r="L5" s="47"/>
     </row>
-    <row r="6" spans="1:12" ht="14.4">
-      <c r="A6" s="141" t="s">
+    <row r="6" spans="1:12" ht="14.25">
+      <c r="A6" s="112" t="s">
         <v>90</v>
       </c>
-      <c r="B6" s="142"/>
+      <c r="B6" s="113"/>
       <c r="C6" s="46" t="s">
         <v>91</v>
       </c>
@@ -2708,11 +2711,11 @@
       <c r="K6" s="40"/>
       <c r="L6" s="44"/>
     </row>
-    <row r="7" spans="1:12" ht="14.4">
-      <c r="A7" s="141" t="s">
+    <row r="7" spans="1:12" ht="14.25">
+      <c r="A7" s="112" t="s">
         <v>92</v>
       </c>
-      <c r="B7" s="142"/>
+      <c r="B7" s="113"/>
       <c r="C7" s="46" t="s">
         <v>93</v>
       </c>
@@ -2726,11 +2729,11 @@
       <c r="K7" s="40"/>
       <c r="L7" s="44"/>
     </row>
-    <row r="8" spans="1:12" ht="14.4">
-      <c r="A8" s="141" t="s">
+    <row r="8" spans="1:12" ht="14.25">
+      <c r="A8" s="112" t="s">
         <v>94</v>
       </c>
-      <c r="B8" s="142"/>
+      <c r="B8" s="113"/>
       <c r="C8" s="46" t="s">
         <v>95</v>
       </c>
@@ -2744,7 +2747,7 @@
       <c r="K8" s="40"/>
       <c r="L8" s="44"/>
     </row>
-    <row r="9" spans="1:12" ht="14.4">
+    <row r="9" spans="1:12" ht="14.25">
       <c r="A9" s="41"/>
       <c r="B9" s="41"/>
       <c r="C9" s="46"/>
@@ -2758,7 +2761,7 @@
       <c r="K9" s="40"/>
       <c r="L9" s="48"/>
     </row>
-    <row r="10" spans="1:12" ht="49.2" customHeight="1">
+    <row r="10" spans="1:12" ht="49.15" customHeight="1">
       <c r="A10" s="49" t="s">
         <v>3</v>
       </c>
@@ -2796,7 +2799,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="11" spans="1:12" s="54" customFormat="1" ht="32.4" customHeight="1">
+    <row r="11" spans="1:12" s="54" customFormat="1" ht="32.450000000000003" customHeight="1">
       <c r="A11" s="51" t="s">
         <v>107</v>
       </c>
@@ -2813,7 +2816,7 @@
       <c r="L11" s="53"/>
     </row>
     <row r="12" spans="1:12" ht="15" customHeight="1">
-      <c r="A12" s="128" t="s">
+      <c r="A12" s="116" t="s">
         <v>108</v>
       </c>
       <c r="B12" s="55" t="s">
@@ -2847,13 +2850,13 @@
         <f t="shared" ref="K12:K65" si="0">I12*J12</f>
         <v>9</v>
       </c>
-      <c r="L12" s="130">
+      <c r="L12" s="118">
         <f>SUM(K12:K18)</f>
         <v>63</v>
       </c>
     </row>
     <row r="13" spans="1:12" ht="15" customHeight="1">
-      <c r="A13" s="129"/>
+      <c r="A13" s="117"/>
       <c r="B13" s="55" t="s">
         <v>113</v>
       </c>
@@ -2885,10 +2888,10 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="L13" s="131"/>
+      <c r="L13" s="119"/>
     </row>
     <row r="14" spans="1:12" ht="15" customHeight="1">
-      <c r="A14" s="129"/>
+      <c r="A14" s="117"/>
       <c r="B14" s="55" t="s">
         <v>116</v>
       </c>
@@ -2920,10 +2923,10 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="L14" s="131"/>
+      <c r="L14" s="119"/>
     </row>
     <row r="15" spans="1:12" ht="15" customHeight="1">
-      <c r="A15" s="129"/>
+      <c r="A15" s="117"/>
       <c r="B15" s="55" t="s">
         <v>119</v>
       </c>
@@ -2955,10 +2958,10 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="L15" s="131"/>
+      <c r="L15" s="119"/>
     </row>
     <row r="16" spans="1:12" ht="15" customHeight="1">
-      <c r="A16" s="129"/>
+      <c r="A16" s="117"/>
       <c r="B16" s="55" t="s">
         <v>122</v>
       </c>
@@ -2990,10 +2993,10 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="L16" s="131"/>
+      <c r="L16" s="119"/>
     </row>
     <row r="17" spans="1:12" ht="15" customHeight="1">
-      <c r="A17" s="129"/>
+      <c r="A17" s="117"/>
       <c r="B17" s="55" t="s">
         <v>125</v>
       </c>
@@ -3025,10 +3028,10 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="L17" s="131"/>
+      <c r="L17" s="119"/>
     </row>
     <row r="18" spans="1:12" ht="15" customHeight="1">
-      <c r="A18" s="129"/>
+      <c r="A18" s="117"/>
       <c r="B18" s="55" t="s">
         <v>128</v>
       </c>
@@ -3060,10 +3063,10 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="L18" s="131"/>
+      <c r="L18" s="119"/>
     </row>
     <row r="19" spans="1:12" ht="15" customHeight="1">
-      <c r="A19" s="132" t="s">
+      <c r="A19" s="120" t="s">
         <v>130</v>
       </c>
       <c r="B19" s="60" t="s">
@@ -3097,13 +3100,13 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="L19" s="134">
+      <c r="L19" s="122">
         <f>SUM(K19:K21)</f>
         <v>27</v>
       </c>
     </row>
     <row r="20" spans="1:12" ht="15" customHeight="1">
-      <c r="A20" s="132"/>
+      <c r="A20" s="120"/>
       <c r="B20" s="60" t="s">
         <v>134</v>
       </c>
@@ -3135,10 +3138,10 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="L20" s="134"/>
+      <c r="L20" s="122"/>
     </row>
     <row r="21" spans="1:12" ht="15" customHeight="1">
-      <c r="A21" s="133"/>
+      <c r="A21" s="121"/>
       <c r="B21" s="60" t="s">
         <v>136</v>
       </c>
@@ -3170,10 +3173,10 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="L21" s="135"/>
+      <c r="L21" s="123"/>
     </row>
     <row r="22" spans="1:12" ht="15" customHeight="1">
-      <c r="A22" s="136" t="s">
+      <c r="A22" s="124" t="s">
         <v>138</v>
       </c>
       <c r="B22" s="65" t="s">
@@ -3207,13 +3210,13 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="L22" s="138">
+      <c r="L22" s="126">
         <f>SUM(K22:K30)</f>
         <v>81</v>
       </c>
     </row>
     <row r="23" spans="1:12" ht="15" customHeight="1">
-      <c r="A23" s="137"/>
+      <c r="A23" s="125"/>
       <c r="B23" s="65" t="s">
         <v>141</v>
       </c>
@@ -3245,10 +3248,10 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="L23" s="139"/>
+      <c r="L23" s="127"/>
     </row>
     <row r="24" spans="1:12" ht="15" customHeight="1">
-      <c r="A24" s="137"/>
+      <c r="A24" s="125"/>
       <c r="B24" s="65" t="s">
         <v>143</v>
       </c>
@@ -3280,10 +3283,10 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="L24" s="139"/>
+      <c r="L24" s="127"/>
     </row>
     <row r="25" spans="1:12" ht="15" customHeight="1">
-      <c r="A25" s="137"/>
+      <c r="A25" s="125"/>
       <c r="B25" s="65" t="s">
         <v>145</v>
       </c>
@@ -3315,10 +3318,10 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="L25" s="139"/>
+      <c r="L25" s="127"/>
     </row>
     <row r="26" spans="1:12" ht="15" customHeight="1">
-      <c r="A26" s="137"/>
+      <c r="A26" s="125"/>
       <c r="B26" s="65" t="s">
         <v>147</v>
       </c>
@@ -3350,10 +3353,10 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="L26" s="139"/>
+      <c r="L26" s="127"/>
     </row>
     <row r="27" spans="1:12" ht="15" customHeight="1">
-      <c r="A27" s="137"/>
+      <c r="A27" s="125"/>
       <c r="B27" s="65" t="s">
         <v>149</v>
       </c>
@@ -3385,10 +3388,10 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="L27" s="139"/>
+      <c r="L27" s="127"/>
     </row>
     <row r="28" spans="1:12" ht="15" customHeight="1">
-      <c r="A28" s="137"/>
+      <c r="A28" s="125"/>
       <c r="B28" s="65" t="s">
         <v>152</v>
       </c>
@@ -3420,10 +3423,10 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="L28" s="139"/>
+      <c r="L28" s="127"/>
     </row>
     <row r="29" spans="1:12" ht="15" customHeight="1">
-      <c r="A29" s="137"/>
+      <c r="A29" s="125"/>
       <c r="B29" s="65" t="s">
         <v>154</v>
       </c>
@@ -3455,10 +3458,10 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="L29" s="139"/>
+      <c r="L29" s="127"/>
     </row>
     <row r="30" spans="1:12" ht="15" customHeight="1">
-      <c r="A30" s="137"/>
+      <c r="A30" s="125"/>
       <c r="B30" s="65" t="s">
         <v>156</v>
       </c>
@@ -3490,10 +3493,10 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="L30" s="139"/>
+      <c r="L30" s="127"/>
     </row>
     <row r="31" spans="1:12" ht="15" customHeight="1">
-      <c r="A31" s="122" t="s">
+      <c r="A31" s="128" t="s">
         <v>158</v>
       </c>
       <c r="B31" s="70" t="s">
@@ -3527,13 +3530,13 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="L31" s="124">
+      <c r="L31" s="130">
         <f>SUM(K31:K44)</f>
         <v>126</v>
       </c>
     </row>
     <row r="32" spans="1:12" ht="15" customHeight="1">
-      <c r="A32" s="122"/>
+      <c r="A32" s="128"/>
       <c r="B32" s="70" t="s">
         <v>161</v>
       </c>
@@ -3565,10 +3568,10 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="L32" s="124"/>
+      <c r="L32" s="130"/>
     </row>
     <row r="33" spans="1:12" ht="15" customHeight="1">
-      <c r="A33" s="122"/>
+      <c r="A33" s="128"/>
       <c r="B33" s="70" t="s">
         <v>163</v>
       </c>
@@ -3600,10 +3603,10 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="L33" s="124"/>
+      <c r="L33" s="130"/>
     </row>
     <row r="34" spans="1:12" ht="15" customHeight="1">
-      <c r="A34" s="123"/>
+      <c r="A34" s="129"/>
       <c r="B34" s="70" t="s">
         <v>165</v>
       </c>
@@ -3635,10 +3638,10 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="L34" s="125"/>
+      <c r="L34" s="131"/>
     </row>
     <row r="35" spans="1:12" ht="15" customHeight="1">
-      <c r="A35" s="123"/>
+      <c r="A35" s="129"/>
       <c r="B35" s="70" t="s">
         <v>167</v>
       </c>
@@ -3670,10 +3673,10 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="L35" s="125"/>
+      <c r="L35" s="131"/>
     </row>
     <row r="36" spans="1:12" ht="15" customHeight="1">
-      <c r="A36" s="123"/>
+      <c r="A36" s="129"/>
       <c r="B36" s="70" t="s">
         <v>169</v>
       </c>
@@ -3705,10 +3708,10 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="L36" s="125"/>
+      <c r="L36" s="131"/>
     </row>
     <row r="37" spans="1:12" ht="15" customHeight="1">
-      <c r="A37" s="123"/>
+      <c r="A37" s="129"/>
       <c r="B37" s="70" t="s">
         <v>171</v>
       </c>
@@ -3740,10 +3743,10 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="L37" s="125"/>
+      <c r="L37" s="131"/>
     </row>
     <row r="38" spans="1:12" ht="15" customHeight="1">
-      <c r="A38" s="123"/>
+      <c r="A38" s="129"/>
       <c r="B38" s="70" t="s">
         <v>173</v>
       </c>
@@ -3775,10 +3778,10 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="L38" s="125"/>
+      <c r="L38" s="131"/>
     </row>
     <row r="39" spans="1:12" ht="15" customHeight="1">
-      <c r="A39" s="123"/>
+      <c r="A39" s="129"/>
       <c r="B39" s="70" t="s">
         <v>176</v>
       </c>
@@ -3810,10 +3813,10 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="L39" s="125"/>
+      <c r="L39" s="131"/>
     </row>
     <row r="40" spans="1:12" ht="15" customHeight="1">
-      <c r="A40" s="123"/>
+      <c r="A40" s="129"/>
       <c r="B40" s="70" t="s">
         <v>178</v>
       </c>
@@ -3845,10 +3848,10 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="L40" s="125"/>
+      <c r="L40" s="131"/>
     </row>
     <row r="41" spans="1:12" ht="15" customHeight="1">
-      <c r="A41" s="123"/>
+      <c r="A41" s="129"/>
       <c r="B41" s="70" t="s">
         <v>180</v>
       </c>
@@ -3880,10 +3883,10 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="L41" s="125"/>
+      <c r="L41" s="131"/>
     </row>
     <row r="42" spans="1:12" ht="15" customHeight="1">
-      <c r="A42" s="123"/>
+      <c r="A42" s="129"/>
       <c r="B42" s="70" t="s">
         <v>182</v>
       </c>
@@ -3915,10 +3918,10 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="L42" s="125"/>
+      <c r="L42" s="131"/>
     </row>
     <row r="43" spans="1:12" ht="15" customHeight="1">
-      <c r="A43" s="123"/>
+      <c r="A43" s="129"/>
       <c r="B43" s="70" t="s">
         <v>184</v>
       </c>
@@ -3950,10 +3953,10 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="L43" s="125"/>
+      <c r="L43" s="131"/>
     </row>
     <row r="44" spans="1:12" ht="15" customHeight="1">
-      <c r="A44" s="123"/>
+      <c r="A44" s="129"/>
       <c r="B44" s="70" t="s">
         <v>185</v>
       </c>
@@ -3985,10 +3988,10 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="L44" s="125"/>
+      <c r="L44" s="131"/>
     </row>
     <row r="45" spans="1:12" ht="15" customHeight="1">
-      <c r="A45" s="126" t="s">
+      <c r="A45" s="132" t="s">
         <v>187</v>
       </c>
       <c r="B45" s="55" t="s">
@@ -4022,13 +4025,13 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="L45" s="127">
+      <c r="L45" s="133">
         <f>SUM(K45:K61)</f>
         <v>153</v>
       </c>
     </row>
     <row r="46" spans="1:12" ht="15" customHeight="1">
-      <c r="A46" s="126"/>
+      <c r="A46" s="132"/>
       <c r="B46" s="55" t="s">
         <v>191</v>
       </c>
@@ -4060,10 +4063,10 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="L46" s="127"/>
+      <c r="L46" s="133"/>
     </row>
     <row r="47" spans="1:12" ht="15" customHeight="1">
-      <c r="A47" s="126"/>
+      <c r="A47" s="132"/>
       <c r="B47" s="55" t="s">
         <v>193</v>
       </c>
@@ -4095,10 +4098,10 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="L47" s="127"/>
+      <c r="L47" s="133"/>
     </row>
     <row r="48" spans="1:12" ht="15" customHeight="1">
-      <c r="A48" s="126"/>
+      <c r="A48" s="132"/>
       <c r="B48" s="55" t="s">
         <v>195</v>
       </c>
@@ -4130,10 +4133,10 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="L48" s="127"/>
+      <c r="L48" s="133"/>
     </row>
     <row r="49" spans="1:12" ht="15" customHeight="1">
-      <c r="A49" s="126"/>
+      <c r="A49" s="132"/>
       <c r="B49" s="55" t="s">
         <v>197</v>
       </c>
@@ -4165,10 +4168,10 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="L49" s="127"/>
+      <c r="L49" s="133"/>
     </row>
     <row r="50" spans="1:12" ht="15" customHeight="1">
-      <c r="A50" s="126"/>
+      <c r="A50" s="132"/>
       <c r="B50" s="55" t="s">
         <v>199</v>
       </c>
@@ -4200,10 +4203,10 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="L50" s="127"/>
+      <c r="L50" s="133"/>
     </row>
     <row r="51" spans="1:12" ht="15" customHeight="1">
-      <c r="A51" s="126"/>
+      <c r="A51" s="132"/>
       <c r="B51" s="55" t="s">
         <v>201</v>
       </c>
@@ -4235,10 +4238,10 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="L51" s="127"/>
+      <c r="L51" s="133"/>
     </row>
     <row r="52" spans="1:12" ht="15" customHeight="1">
-      <c r="A52" s="126"/>
+      <c r="A52" s="132"/>
       <c r="B52" s="55" t="s">
         <v>203</v>
       </c>
@@ -4270,10 +4273,10 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="L52" s="127"/>
+      <c r="L52" s="133"/>
     </row>
     <row r="53" spans="1:12" ht="15" customHeight="1">
-      <c r="A53" s="126"/>
+      <c r="A53" s="132"/>
       <c r="B53" s="55" t="s">
         <v>205</v>
       </c>
@@ -4305,10 +4308,10 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="L53" s="127"/>
+      <c r="L53" s="133"/>
     </row>
     <row r="54" spans="1:12" ht="15" customHeight="1">
-      <c r="A54" s="126"/>
+      <c r="A54" s="132"/>
       <c r="B54" s="55" t="s">
         <v>207</v>
       </c>
@@ -4340,10 +4343,10 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="L54" s="127"/>
+      <c r="L54" s="133"/>
     </row>
     <row r="55" spans="1:12" ht="15" customHeight="1">
-      <c r="A55" s="126"/>
+      <c r="A55" s="132"/>
       <c r="B55" s="55" t="s">
         <v>209</v>
       </c>
@@ -4375,10 +4378,10 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="L55" s="127"/>
+      <c r="L55" s="133"/>
     </row>
     <row r="56" spans="1:12" ht="15" customHeight="1">
-      <c r="A56" s="126"/>
+      <c r="A56" s="132"/>
       <c r="B56" s="55" t="s">
         <v>211</v>
       </c>
@@ -4410,10 +4413,10 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="L56" s="127"/>
+      <c r="L56" s="133"/>
     </row>
     <row r="57" spans="1:12" ht="15" customHeight="1">
-      <c r="A57" s="126"/>
+      <c r="A57" s="132"/>
       <c r="B57" s="55" t="s">
         <v>213</v>
       </c>
@@ -4445,10 +4448,10 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="L57" s="127"/>
+      <c r="L57" s="133"/>
     </row>
     <row r="58" spans="1:12" ht="15" customHeight="1">
-      <c r="A58" s="126"/>
+      <c r="A58" s="132"/>
       <c r="B58" s="55" t="s">
         <v>215</v>
       </c>
@@ -4480,10 +4483,10 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="L58" s="127"/>
+      <c r="L58" s="133"/>
     </row>
     <row r="59" spans="1:12" ht="15" customHeight="1">
-      <c r="A59" s="126"/>
+      <c r="A59" s="132"/>
       <c r="B59" s="55" t="s">
         <v>217</v>
       </c>
@@ -4515,10 +4518,10 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="L59" s="127"/>
+      <c r="L59" s="133"/>
     </row>
     <row r="60" spans="1:12" ht="15" customHeight="1">
-      <c r="A60" s="126"/>
+      <c r="A60" s="132"/>
       <c r="B60" s="55" t="s">
         <v>220</v>
       </c>
@@ -4550,10 +4553,10 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="L60" s="127"/>
+      <c r="L60" s="133"/>
     </row>
     <row r="61" spans="1:12" ht="15" customHeight="1">
-      <c r="A61" s="126"/>
+      <c r="A61" s="132"/>
       <c r="B61" s="55" t="s">
         <v>222</v>
       </c>
@@ -4585,10 +4588,10 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="L61" s="127"/>
+      <c r="L61" s="133"/>
     </row>
     <row r="62" spans="1:12" ht="15" customHeight="1">
-      <c r="A62" s="114" t="s">
+      <c r="A62" s="134" t="s">
         <v>224</v>
       </c>
       <c r="B62" s="76" t="s">
@@ -4622,13 +4625,13 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="L62" s="116">
+      <c r="L62" s="136">
         <f>SUM(K62:K65)</f>
         <v>36</v>
       </c>
     </row>
     <row r="63" spans="1:12" ht="15" customHeight="1">
-      <c r="A63" s="115"/>
+      <c r="A63" s="135"/>
       <c r="B63" s="76" t="s">
         <v>227</v>
       </c>
@@ -4660,10 +4663,10 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="L63" s="117"/>
+      <c r="L63" s="137"/>
     </row>
     <row r="64" spans="1:12" ht="15" customHeight="1">
-      <c r="A64" s="115"/>
+      <c r="A64" s="135"/>
       <c r="B64" s="76" t="s">
         <v>229</v>
       </c>
@@ -4695,10 +4698,10 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="L64" s="117"/>
+      <c r="L64" s="137"/>
     </row>
     <row r="65" spans="1:12" ht="15" customHeight="1">
-      <c r="A65" s="115"/>
+      <c r="A65" s="135"/>
       <c r="B65" s="76" t="s">
         <v>231</v>
       </c>
@@ -4730,7 +4733,7 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="L65" s="117"/>
+      <c r="L65" s="137"/>
     </row>
     <row r="66" spans="1:12" s="54" customFormat="1" ht="27.6" customHeight="1">
       <c r="A66" s="81" t="s">
@@ -4757,7 +4760,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="67" spans="1:12" ht="13.8">
+    <row r="67" spans="1:12" ht="12.75">
       <c r="A67" s="84"/>
       <c r="B67" s="44"/>
       <c r="C67" s="85"/>
@@ -4771,7 +4774,7 @@
       <c r="K67" s="85"/>
       <c r="L67" s="85"/>
     </row>
-    <row r="68" spans="1:12" ht="13.8">
+    <row r="68" spans="1:12" ht="12.75">
       <c r="A68" s="84"/>
       <c r="B68" s="44"/>
       <c r="C68" s="85"/>
@@ -4785,7 +4788,7 @@
       <c r="K68" s="85"/>
       <c r="L68" s="85"/>
     </row>
-    <row r="69" spans="1:12" ht="13.8">
+    <row r="69" spans="1:12" ht="12.75">
       <c r="A69" s="84"/>
       <c r="B69" s="44"/>
       <c r="C69" s="85"/>
@@ -4799,7 +4802,7 @@
       <c r="K69" s="85"/>
       <c r="L69" s="85"/>
     </row>
-    <row r="70" spans="1:12" ht="13.8">
+    <row r="70" spans="1:12" ht="12.75">
       <c r="A70" s="84"/>
       <c r="B70" s="44"/>
       <c r="C70" s="85"/>
@@ -4841,7 +4844,7 @@
       <c r="K72" s="85"/>
       <c r="L72" s="85"/>
     </row>
-    <row r="73" spans="1:12" ht="49.2" customHeight="1">
+    <row r="73" spans="1:12" ht="49.15" customHeight="1">
       <c r="A73" s="49" t="s">
         <v>3</v>
       </c>
@@ -4879,7 +4882,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="74" spans="1:12" s="54" customFormat="1" ht="32.4" customHeight="1">
+    <row r="74" spans="1:12" s="54" customFormat="1" ht="32.450000000000003" customHeight="1">
       <c r="A74" s="86" t="s">
         <v>235</v>
       </c>
@@ -4896,7 +4899,7 @@
       <c r="L74" s="88"/>
     </row>
     <row r="75" spans="1:12" ht="13.35" customHeight="1">
-      <c r="A75" s="112" t="s">
+      <c r="A75" s="138" t="s">
         <v>236</v>
       </c>
       <c r="B75" s="89" t="s">
@@ -4930,13 +4933,13 @@
         <f>I75*J75</f>
         <v>9</v>
       </c>
-      <c r="L75" s="113">
+      <c r="L75" s="139">
         <f>SUM(K75:K103)</f>
         <v>261</v>
       </c>
     </row>
-    <row r="76" spans="1:12" ht="13.2" customHeight="1">
-      <c r="A76" s="112"/>
+    <row r="76" spans="1:12" ht="13.15" customHeight="1">
+      <c r="A76" s="138"/>
       <c r="B76" s="89" t="s">
         <v>240</v>
       </c>
@@ -4968,10 +4971,10 @@
         <f t="shared" ref="K76:K103" si="1">I76*J76</f>
         <v>9</v>
       </c>
-      <c r="L76" s="113"/>
-    </row>
-    <row r="77" spans="1:12" ht="13.2" customHeight="1">
-      <c r="A77" s="112"/>
+      <c r="L76" s="139"/>
+    </row>
+    <row r="77" spans="1:12" ht="13.15" customHeight="1">
+      <c r="A77" s="138"/>
       <c r="B77" s="89" t="s">
         <v>242</v>
       </c>
@@ -5003,10 +5006,10 @@
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="L77" s="113"/>
-    </row>
-    <row r="78" spans="1:12" ht="13.2" customHeight="1">
-      <c r="A78" s="112"/>
+      <c r="L77" s="139"/>
+    </row>
+    <row r="78" spans="1:12" ht="13.15" customHeight="1">
+      <c r="A78" s="138"/>
       <c r="B78" s="89" t="s">
         <v>244</v>
       </c>
@@ -5038,10 +5041,10 @@
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="L78" s="113"/>
-    </row>
-    <row r="79" spans="1:12" ht="13.2" customHeight="1">
-      <c r="A79" s="112"/>
+      <c r="L78" s="139"/>
+    </row>
+    <row r="79" spans="1:12" ht="13.15" customHeight="1">
+      <c r="A79" s="138"/>
       <c r="B79" s="89" t="s">
         <v>246</v>
       </c>
@@ -5073,10 +5076,10 @@
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="L79" s="113"/>
-    </row>
-    <row r="80" spans="1:12" ht="13.2" customHeight="1">
-      <c r="A80" s="112"/>
+      <c r="L79" s="139"/>
+    </row>
+    <row r="80" spans="1:12" ht="13.15" customHeight="1">
+      <c r="A80" s="138"/>
       <c r="B80" s="89" t="s">
         <v>248</v>
       </c>
@@ -5108,10 +5111,10 @@
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="L80" s="113"/>
-    </row>
-    <row r="81" spans="1:12" ht="13.2" customHeight="1">
-      <c r="A81" s="112"/>
+      <c r="L80" s="139"/>
+    </row>
+    <row r="81" spans="1:12" ht="13.15" customHeight="1">
+      <c r="A81" s="138"/>
       <c r="B81" s="89" t="s">
         <v>250</v>
       </c>
@@ -5143,10 +5146,10 @@
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="L81" s="113"/>
-    </row>
-    <row r="82" spans="1:12" ht="13.2" customHeight="1">
-      <c r="A82" s="112"/>
+      <c r="L81" s="139"/>
+    </row>
+    <row r="82" spans="1:12" ht="13.15" customHeight="1">
+      <c r="A82" s="138"/>
       <c r="B82" s="89" t="s">
         <v>252</v>
       </c>
@@ -5178,10 +5181,10 @@
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="L82" s="113"/>
-    </row>
-    <row r="83" spans="1:12" ht="13.2" customHeight="1">
-      <c r="A83" s="112"/>
+      <c r="L82" s="139"/>
+    </row>
+    <row r="83" spans="1:12" ht="13.15" customHeight="1">
+      <c r="A83" s="138"/>
       <c r="B83" s="89" t="s">
         <v>255</v>
       </c>
@@ -5213,10 +5216,10 @@
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="L83" s="113"/>
-    </row>
-    <row r="84" spans="1:12" ht="13.2" customHeight="1">
-      <c r="A84" s="112"/>
+      <c r="L83" s="139"/>
+    </row>
+    <row r="84" spans="1:12" ht="13.15" customHeight="1">
+      <c r="A84" s="138"/>
       <c r="B84" s="89" t="s">
         <v>257</v>
       </c>
@@ -5248,10 +5251,10 @@
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="L84" s="113"/>
-    </row>
-    <row r="85" spans="1:12" ht="13.2" customHeight="1">
-      <c r="A85" s="112"/>
+      <c r="L84" s="139"/>
+    </row>
+    <row r="85" spans="1:12" ht="13.15" customHeight="1">
+      <c r="A85" s="138"/>
       <c r="B85" s="89" t="s">
         <v>259</v>
       </c>
@@ -5283,10 +5286,10 @@
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="L85" s="113"/>
-    </row>
-    <row r="86" spans="1:12" ht="13.2" customHeight="1">
-      <c r="A86" s="112"/>
+      <c r="L85" s="139"/>
+    </row>
+    <row r="86" spans="1:12" ht="13.15" customHeight="1">
+      <c r="A86" s="138"/>
       <c r="B86" s="89" t="s">
         <v>261</v>
       </c>
@@ -5318,10 +5321,10 @@
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="L86" s="113"/>
-    </row>
-    <row r="87" spans="1:12" ht="13.2" customHeight="1">
-      <c r="A87" s="112"/>
+      <c r="L86" s="139"/>
+    </row>
+    <row r="87" spans="1:12" ht="13.15" customHeight="1">
+      <c r="A87" s="138"/>
       <c r="B87" s="89" t="s">
         <v>263</v>
       </c>
@@ -5353,10 +5356,10 @@
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="L87" s="113"/>
-    </row>
-    <row r="88" spans="1:12" ht="13.2" customHeight="1">
-      <c r="A88" s="112"/>
+      <c r="L87" s="139"/>
+    </row>
+    <row r="88" spans="1:12" ht="13.15" customHeight="1">
+      <c r="A88" s="138"/>
       <c r="B88" s="89" t="s">
         <v>265</v>
       </c>
@@ -5388,10 +5391,10 @@
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="L88" s="113"/>
+      <c r="L88" s="139"/>
     </row>
     <row r="89" spans="1:12" ht="15" customHeight="1">
-      <c r="A89" s="112"/>
+      <c r="A89" s="138"/>
       <c r="B89" s="89" t="s">
         <v>267</v>
       </c>
@@ -5423,10 +5426,10 @@
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="L89" s="113"/>
+      <c r="L89" s="139"/>
     </row>
     <row r="90" spans="1:12" ht="15" customHeight="1">
-      <c r="A90" s="112"/>
+      <c r="A90" s="138"/>
       <c r="B90" s="89" t="s">
         <v>270</v>
       </c>
@@ -5458,10 +5461,10 @@
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="L90" s="113"/>
+      <c r="L90" s="139"/>
     </row>
     <row r="91" spans="1:12" ht="15" customHeight="1">
-      <c r="A91" s="112"/>
+      <c r="A91" s="138"/>
       <c r="B91" s="89" t="s">
         <v>272</v>
       </c>
@@ -5493,10 +5496,10 @@
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="L91" s="113"/>
+      <c r="L91" s="139"/>
     </row>
     <row r="92" spans="1:12" ht="15" customHeight="1">
-      <c r="A92" s="112"/>
+      <c r="A92" s="138"/>
       <c r="B92" s="89" t="s">
         <v>274</v>
       </c>
@@ -5528,10 +5531,10 @@
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="L92" s="113"/>
+      <c r="L92" s="139"/>
     </row>
     <row r="93" spans="1:12" ht="15" customHeight="1">
-      <c r="A93" s="112"/>
+      <c r="A93" s="138"/>
       <c r="B93" s="89" t="s">
         <v>276</v>
       </c>
@@ -5563,10 +5566,10 @@
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="L93" s="113"/>
+      <c r="L93" s="139"/>
     </row>
     <row r="94" spans="1:12" ht="15" customHeight="1">
-      <c r="A94" s="112"/>
+      <c r="A94" s="138"/>
       <c r="B94" s="89" t="s">
         <v>278</v>
       </c>
@@ -5598,10 +5601,10 @@
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="L94" s="113"/>
+      <c r="L94" s="139"/>
     </row>
     <row r="95" spans="1:12" ht="15" customHeight="1">
-      <c r="A95" s="112"/>
+      <c r="A95" s="138"/>
       <c r="B95" s="89" t="s">
         <v>280</v>
       </c>
@@ -5633,10 +5636,10 @@
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="L95" s="113"/>
+      <c r="L95" s="139"/>
     </row>
     <row r="96" spans="1:12" ht="15" customHeight="1">
-      <c r="A96" s="112"/>
+      <c r="A96" s="138"/>
       <c r="B96" s="89" t="s">
         <v>282</v>
       </c>
@@ -5668,10 +5671,10 @@
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="L96" s="113"/>
+      <c r="L96" s="139"/>
     </row>
     <row r="97" spans="1:12" ht="15" customHeight="1">
-      <c r="A97" s="112"/>
+      <c r="A97" s="138"/>
       <c r="B97" s="89" t="s">
         <v>284</v>
       </c>
@@ -5703,10 +5706,10 @@
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="L97" s="113"/>
+      <c r="L97" s="139"/>
     </row>
     <row r="98" spans="1:12" ht="15" customHeight="1">
-      <c r="A98" s="112"/>
+      <c r="A98" s="138"/>
       <c r="B98" s="89" t="s">
         <v>286</v>
       </c>
@@ -5738,10 +5741,10 @@
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="L98" s="113"/>
+      <c r="L98" s="139"/>
     </row>
     <row r="99" spans="1:12" ht="15" customHeight="1">
-      <c r="A99" s="112"/>
+      <c r="A99" s="138"/>
       <c r="B99" s="89" t="s">
         <v>288</v>
       </c>
@@ -5773,10 +5776,10 @@
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="L99" s="113"/>
+      <c r="L99" s="139"/>
     </row>
     <row r="100" spans="1:12" ht="15" customHeight="1">
-      <c r="A100" s="112"/>
+      <c r="A100" s="138"/>
       <c r="B100" s="89" t="s">
         <v>290</v>
       </c>
@@ -5808,10 +5811,10 @@
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="L100" s="113"/>
+      <c r="L100" s="139"/>
     </row>
     <row r="101" spans="1:12" ht="15" customHeight="1">
-      <c r="A101" s="112"/>
+      <c r="A101" s="138"/>
       <c r="B101" s="89" t="s">
         <v>293</v>
       </c>
@@ -5843,10 +5846,10 @@
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="L101" s="113"/>
+      <c r="L101" s="139"/>
     </row>
     <row r="102" spans="1:12" ht="15" customHeight="1">
-      <c r="A102" s="112"/>
+      <c r="A102" s="138"/>
       <c r="B102" s="89" t="s">
         <v>295</v>
       </c>
@@ -5878,10 +5881,10 @@
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="L102" s="113"/>
+      <c r="L102" s="139"/>
     </row>
     <row r="103" spans="1:12" ht="15" customHeight="1">
-      <c r="A103" s="112"/>
+      <c r="A103" s="138"/>
       <c r="B103" s="89" t="s">
         <v>297</v>
       </c>
@@ -5913,9 +5916,9 @@
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="L103" s="113"/>
-    </row>
-    <row r="104" spans="1:12" s="54" customFormat="1" ht="34.200000000000003" customHeight="1">
+      <c r="L103" s="139"/>
+    </row>
+    <row r="104" spans="1:12" s="54" customFormat="1" ht="34.15" customHeight="1">
       <c r="A104" s="94"/>
       <c r="B104" s="95"/>
       <c r="C104" s="95"/>
@@ -5929,7 +5932,7 @@
       <c r="K104" s="95"/>
       <c r="L104" s="97"/>
     </row>
-    <row r="105" spans="1:12" s="54" customFormat="1" ht="44.4" customHeight="1">
+    <row r="105" spans="1:12" s="54" customFormat="1" ht="44.45" customHeight="1">
       <c r="A105" s="94"/>
       <c r="B105" s="95"/>
       <c r="C105" s="95"/>
@@ -5944,7 +5947,7 @@
       <c r="L105" s="97"/>
     </row>
     <row r="106" spans="1:12" ht="15" customHeight="1">
-      <c r="A106" s="114" t="s">
+      <c r="A106" s="134" t="s">
         <v>299</v>
       </c>
       <c r="B106" s="76" t="s">
@@ -5978,13 +5981,13 @@
         <f t="shared" ref="K106:K112" si="2">I106*J106</f>
         <v>9</v>
       </c>
-      <c r="L106" s="116">
+      <c r="L106" s="136">
         <f>SUM(K106:K109)</f>
         <v>36</v>
       </c>
     </row>
     <row r="107" spans="1:12" ht="15" customHeight="1">
-      <c r="A107" s="115"/>
+      <c r="A107" s="135"/>
       <c r="B107" s="76" t="s">
         <v>301</v>
       </c>
@@ -6016,10 +6019,10 @@
         <f t="shared" si="2"/>
         <v>9</v>
       </c>
-      <c r="L107" s="117"/>
+      <c r="L107" s="137"/>
     </row>
     <row r="108" spans="1:12" ht="15" customHeight="1">
-      <c r="A108" s="115"/>
+      <c r="A108" s="135"/>
       <c r="B108" s="76" t="s">
         <v>302</v>
       </c>
@@ -6051,10 +6054,10 @@
         <f t="shared" si="2"/>
         <v>9</v>
       </c>
-      <c r="L108" s="117"/>
+      <c r="L108" s="137"/>
     </row>
     <row r="109" spans="1:12" ht="15" customHeight="1">
-      <c r="A109" s="115"/>
+      <c r="A109" s="135"/>
       <c r="B109" s="76" t="s">
         <v>304</v>
       </c>
@@ -6086,10 +6089,10 @@
         <f t="shared" si="2"/>
         <v>9</v>
       </c>
-      <c r="L109" s="117"/>
+      <c r="L109" s="137"/>
     </row>
     <row r="110" spans="1:12" ht="15" customHeight="1">
-      <c r="A110" s="118" t="s">
+      <c r="A110" s="140" t="s">
         <v>306</v>
       </c>
       <c r="B110" s="98" t="s">
@@ -6123,13 +6126,13 @@
         <f t="shared" si="2"/>
         <v>9</v>
       </c>
-      <c r="L110" s="120">
+      <c r="L110" s="142">
         <f>SUM(K110:K112)</f>
         <v>27</v>
       </c>
     </row>
     <row r="111" spans="1:12" ht="15" customHeight="1">
-      <c r="A111" s="119"/>
+      <c r="A111" s="141"/>
       <c r="B111" s="98" t="s">
         <v>310</v>
       </c>
@@ -6161,10 +6164,10 @@
         <f t="shared" si="2"/>
         <v>9</v>
       </c>
-      <c r="L111" s="121"/>
+      <c r="L111" s="143"/>
     </row>
     <row r="112" spans="1:12" ht="15" customHeight="1">
-      <c r="A112" s="119"/>
+      <c r="A112" s="141"/>
       <c r="B112" s="98" t="s">
         <v>312</v>
       </c>
@@ -6196,7 +6199,7 @@
         <f t="shared" si="2"/>
         <v>9</v>
       </c>
-      <c r="L112" s="121"/>
+      <c r="L112" s="143"/>
     </row>
     <row r="113" spans="1:12" s="54" customFormat="1" ht="27.6" customHeight="1">
       <c r="A113" s="81" t="s">
@@ -6223,7 +6226,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="114" spans="1:12" ht="13.8">
+    <row r="114" spans="1:12" ht="12.75">
       <c r="A114" s="40"/>
       <c r="B114" s="44"/>
       <c r="C114" s="40"/>
@@ -6237,7 +6240,7 @@
       <c r="K114" s="40"/>
       <c r="L114" s="44"/>
     </row>
-    <row r="115" spans="1:12" ht="46.2" customHeight="1">
+    <row r="115" spans="1:12" ht="46.15" customHeight="1">
       <c r="A115" s="40"/>
       <c r="B115" s="44"/>
       <c r="C115" s="40"/>
@@ -6251,7 +6254,7 @@
       <c r="K115" s="40"/>
       <c r="L115" s="44"/>
     </row>
-    <row r="116" spans="1:12" ht="14.4">
+    <row r="116" spans="1:12" ht="14.25">
       <c r="A116" s="103"/>
       <c r="B116" s="48" t="s">
         <v>314</v>
@@ -6269,7 +6272,7 @@
       <c r="K116" s="103"/>
       <c r="L116" s="104"/>
     </row>
-    <row r="117" spans="1:12" ht="14.4">
+    <row r="117" spans="1:12" ht="14.25">
       <c r="A117" s="103"/>
       <c r="B117" s="48" t="s">
         <v>316</v>
@@ -6287,7 +6290,7 @@
       <c r="K117" s="103"/>
       <c r="L117" s="104"/>
     </row>
-    <row r="118" spans="1:12" ht="14.4">
+    <row r="118" spans="1:12" ht="15">
       <c r="A118" s="103"/>
       <c r="B118" s="105"/>
       <c r="C118" s="103"/>
@@ -6301,7 +6304,7 @@
       <c r="K118" s="103"/>
       <c r="L118" s="104"/>
     </row>
-    <row r="119" spans="1:12" ht="14.4">
+    <row r="119" spans="1:12" ht="14.25">
       <c r="A119" s="103"/>
       <c r="B119" s="48"/>
       <c r="C119" s="103"/>
@@ -6315,7 +6318,7 @@
       <c r="K119" s="103"/>
       <c r="L119" s="104"/>
     </row>
-    <row r="120" spans="1:12" ht="14.4">
+    <row r="120" spans="1:12" ht="14.25">
       <c r="A120" s="103"/>
       <c r="B120" s="48"/>
       <c r="C120" s="103"/>
@@ -6329,7 +6332,7 @@
       <c r="K120" s="103"/>
       <c r="L120" s="104"/>
     </row>
-    <row r="121" spans="1:12" ht="14.4">
+    <row r="121" spans="1:12" ht="15">
       <c r="A121" s="103"/>
       <c r="B121" s="107" t="s">
         <v>318</v>
@@ -6347,7 +6350,7 @@
       <c r="K121" s="103"/>
       <c r="L121" s="104"/>
     </row>
-    <row r="122" spans="1:12" ht="14.4">
+    <row r="122" spans="1:12" ht="14.25">
       <c r="A122" s="103"/>
       <c r="B122" s="48" t="s">
         <v>320</v>
@@ -6403,30 +6406,30 @@
     </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="A75:A103"/>
+    <mergeCell ref="L75:L103"/>
+    <mergeCell ref="A106:A109"/>
+    <mergeCell ref="L106:L109"/>
+    <mergeCell ref="A110:A112"/>
+    <mergeCell ref="L110:L112"/>
+    <mergeCell ref="A31:A44"/>
+    <mergeCell ref="L31:L44"/>
+    <mergeCell ref="A45:A61"/>
+    <mergeCell ref="L45:L61"/>
+    <mergeCell ref="A62:A65"/>
+    <mergeCell ref="L62:L65"/>
+    <mergeCell ref="A12:A18"/>
+    <mergeCell ref="L12:L18"/>
+    <mergeCell ref="A19:A21"/>
+    <mergeCell ref="L19:L21"/>
+    <mergeCell ref="A22:A30"/>
+    <mergeCell ref="L22:L30"/>
     <mergeCell ref="A8:B8"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C5:D5"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="A7:B7"/>
-    <mergeCell ref="A12:A18"/>
-    <mergeCell ref="L12:L18"/>
-    <mergeCell ref="A19:A21"/>
-    <mergeCell ref="L19:L21"/>
-    <mergeCell ref="A22:A30"/>
-    <mergeCell ref="L22:L30"/>
-    <mergeCell ref="A31:A44"/>
-    <mergeCell ref="L31:L44"/>
-    <mergeCell ref="A45:A61"/>
-    <mergeCell ref="L45:L61"/>
-    <mergeCell ref="A62:A65"/>
-    <mergeCell ref="L62:L65"/>
-    <mergeCell ref="A75:A103"/>
-    <mergeCell ref="L75:L103"/>
-    <mergeCell ref="A106:A109"/>
-    <mergeCell ref="L106:L109"/>
-    <mergeCell ref="A110:A112"/>
-    <mergeCell ref="L110:L112"/>
   </mergeCells>
   <pageMargins left="0.15" right="0.12" top="0.24" bottom="0.23" header="0.14000000000000001" footer="0.15"/>
   <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
@@ -6437,22 +6440,22 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:X1005"/>
-  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="7.109375" customWidth="1"/>
-    <col min="2" max="2" width="19.109375" customWidth="1"/>
-    <col min="3" max="3" width="16.109375" customWidth="1"/>
-    <col min="4" max="4" width="15.6640625" customWidth="1"/>
-    <col min="5" max="5" width="13.33203125" customWidth="1"/>
-    <col min="6" max="6" width="15.5546875" customWidth="1"/>
-    <col min="7" max="7" width="16.88671875" customWidth="1"/>
-    <col min="8" max="8" width="11.33203125" customWidth="1"/>
-    <col min="9" max="9" width="7.88671875" customWidth="1"/>
-    <col min="10" max="12" width="11.33203125" customWidth="1"/>
-    <col min="13" max="24" width="8.6640625" customWidth="1"/>
+    <col min="1" max="1" width="7.140625" customWidth="1"/>
+    <col min="2" max="2" width="19.140625" customWidth="1"/>
+    <col min="3" max="3" width="16.140625" customWidth="1"/>
+    <col min="4" max="4" width="15.7109375" customWidth="1"/>
+    <col min="5" max="5" width="13.28515625" customWidth="1"/>
+    <col min="6" max="6" width="15.5703125" customWidth="1"/>
+    <col min="7" max="7" width="16.85546875" customWidth="1"/>
+    <col min="8" max="8" width="11.28515625" customWidth="1"/>
+    <col min="9" max="9" width="7.85546875" customWidth="1"/>
+    <col min="10" max="12" width="11.28515625" customWidth="1"/>
+    <col min="13" max="24" width="8.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" ht="18">
+    <row r="1" spans="1:24" ht="18.75">
       <c r="A1" s="144" t="s">
         <v>1</v>
       </c>
@@ -6480,7 +6483,7 @@
       <c r="W1" s="1"/>
       <c r="X1" s="1"/>
     </row>
-    <row r="2" spans="1:24" ht="15.6">
+    <row r="2" spans="1:24" ht="15.75">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -6506,7 +6509,7 @@
       <c r="W2" s="1"/>
       <c r="X2" s="1"/>
     </row>
-    <row r="3" spans="1:24" ht="15.6">
+    <row r="3" spans="1:24" ht="15.75">
       <c r="A3" s="4" t="s">
         <v>2</v>
       </c>
@@ -6536,7 +6539,7 @@
       <c r="W3" s="1"/>
       <c r="X3" s="1"/>
     </row>
-    <row r="4" spans="1:24" ht="15.6">
+    <row r="4" spans="1:24" ht="15.75">
       <c r="A4" s="4" t="s">
         <v>5</v>
       </c>
@@ -6566,7 +6569,7 @@
       <c r="W4" s="1"/>
       <c r="X4" s="1"/>
     </row>
-    <row r="5" spans="1:24" ht="15.6">
+    <row r="5" spans="1:24" ht="15.75">
       <c r="A5" s="4" t="s">
         <v>7</v>
       </c>
@@ -6596,7 +6599,7 @@
       <c r="W5" s="1"/>
       <c r="X5" s="1"/>
     </row>
-    <row r="6" spans="1:24" ht="15.6">
+    <row r="6" spans="1:24" ht="15.75">
       <c r="A6" s="4" t="s">
         <v>9</v>
       </c>
@@ -6626,7 +6629,7 @@
       <c r="W6" s="1"/>
       <c r="X6" s="1"/>
     </row>
-    <row r="7" spans="1:24" ht="15.6">
+    <row r="7" spans="1:24" ht="15.75">
       <c r="A7" s="4" t="s">
         <v>11</v>
       </c>
@@ -6656,7 +6659,7 @@
       <c r="W7" s="1"/>
       <c r="X7" s="1"/>
     </row>
-    <row r="8" spans="1:24" ht="15.6">
+    <row r="8" spans="1:24" ht="15.75">
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
@@ -6682,7 +6685,7 @@
       <c r="W8" s="1"/>
       <c r="X8" s="1"/>
     </row>
-    <row r="9" spans="1:24" ht="15.6">
+    <row r="9" spans="1:24" ht="15.75">
       <c r="A9" s="146" t="s">
         <v>3</v>
       </c>
@@ -32803,17 +32806,17 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:Z1007"/>
-  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="8.88671875" customWidth="1"/>
-    <col min="2" max="2" width="21.6640625" customWidth="1"/>
+    <col min="1" max="1" width="8.85546875" customWidth="1"/>
+    <col min="2" max="2" width="21.7109375" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
-    <col min="4" max="4" width="36.5546875" customWidth="1"/>
-    <col min="5" max="9" width="13.33203125" customWidth="1"/>
-    <col min="10" max="26" width="8.6640625" customWidth="1"/>
+    <col min="4" max="4" width="36.5703125" customWidth="1"/>
+    <col min="5" max="9" width="13.28515625" customWidth="1"/>
+    <col min="10" max="26" width="8.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" ht="14.4">
+    <row r="1" spans="1:26">
       <c r="A1" s="150" t="s">
         <v>0</v>
       </c>
@@ -32843,7 +32846,7 @@
       <c r="Y1" s="5"/>
       <c r="Z1" s="5"/>
     </row>
-    <row r="2" spans="1:26" ht="15.6">
+    <row r="2" spans="1:26" ht="15.75">
       <c r="A2" s="4"/>
       <c r="B2" s="2"/>
       <c r="C2" s="4"/>
@@ -32871,13 +32874,13 @@
       <c r="Y2" s="5"/>
       <c r="Z2" s="5"/>
     </row>
-    <row r="3" spans="1:26" ht="15.6">
+    <row r="3" spans="1:26" ht="15.75">
       <c r="A3" s="4" t="s">
         <v>2</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="4" t="s">
-        <v>4</v>
+        <v>322</v>
       </c>
       <c r="D3" s="3"/>
       <c r="E3" s="6"/>
@@ -32903,7 +32906,7 @@
       <c r="Y3" s="5"/>
       <c r="Z3" s="5"/>
     </row>
-    <row r="4" spans="1:26" ht="15.6">
+    <row r="4" spans="1:26" ht="15.75">
       <c r="A4" s="4" t="s">
         <v>5</v>
       </c>
@@ -32935,7 +32938,7 @@
       <c r="Y4" s="5"/>
       <c r="Z4" s="5"/>
     </row>
-    <row r="5" spans="1:26" ht="15.6">
+    <row r="5" spans="1:26" ht="15.75">
       <c r="A5" s="4" t="s">
         <v>7</v>
       </c>
@@ -32967,7 +32970,7 @@
       <c r="Y5" s="5"/>
       <c r="Z5" s="5"/>
     </row>
-    <row r="6" spans="1:26" ht="15.6">
+    <row r="6" spans="1:26" ht="15.75">
       <c r="A6" s="4" t="s">
         <v>81</v>
       </c>
@@ -32999,7 +33002,7 @@
       <c r="Y6" s="5"/>
       <c r="Z6" s="5"/>
     </row>
-    <row r="7" spans="1:26" ht="15.6">
+    <row r="7" spans="1:26" ht="15.75">
       <c r="A7" s="4" t="s">
         <v>11</v>
       </c>
@@ -33031,7 +33034,7 @@
       <c r="Y7" s="5"/>
       <c r="Z7" s="5"/>
     </row>
-    <row r="8" spans="1:26" ht="15.6">
+    <row r="8" spans="1:26" ht="15.75">
       <c r="A8" s="4"/>
       <c r="B8" s="2"/>
       <c r="C8" s="4"/>
@@ -33059,7 +33062,7 @@
       <c r="Y8" s="5"/>
       <c r="Z8" s="5"/>
     </row>
-    <row r="9" spans="1:26" ht="14.4">
+    <row r="9" spans="1:26">
       <c r="A9" s="151" t="s">
         <v>3</v>
       </c>
@@ -33414,7 +33417,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="24" spans="1:9" ht="14.4">
+    <row r="24" spans="1:9">
       <c r="A24" s="30">
         <v>11</v>
       </c>
@@ -33439,7 +33442,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="25" spans="1:9" ht="14.4">
+    <row r="25" spans="1:9">
       <c r="A25" s="30">
         <v>12</v>
       </c>
@@ -33454,14 +33457,14 @@
         <v>73</v>
       </c>
     </row>
-    <row r="26" spans="1:9" ht="14.4">
+    <row r="26" spans="1:9">
       <c r="A26" s="13"/>
       <c r="I26" s="8">
         <f>COUNTIF(I11:I25, "sudah")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:9" ht="14.4">
+    <row r="27" spans="1:9">
       <c r="A27" s="13"/>
       <c r="I27" s="8">
         <f>COUNTA(B11:B25)</f>

</xml_diff>